<commit_message>
ci/cd: update test cases excel reports with description column, non-fatal auth fixes, and workflow updates
</commit_message>
<xml_diff>
--- a/automation/reports/Excel/Failed_Test_Cases.xlsx
+++ b/automation/reports/Excel/Failed_Test_Cases.xlsx
@@ -46,7 +46,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -54,13 +54,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -428,19 +442,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Test ID</t>
@@ -448,30 +463,35 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Module</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Execution Time (s)</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Failure Reason</t>
         </is>

</xml_diff>